<commit_message>
Update suite aux reviews ec271c51cfb6c24690a83201d38b9a8e70431e88
</commit_message>
<xml_diff>
--- a/htr-Mapping-CDA-FHIR/ig/StructureDefinition-EnteteDocument.xlsx
+++ b/htr-Mapping-CDA-FHIR/ig/StructureDefinition-EnteteDocument.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-21T13:48:36+00:00</t>
+    <t>2025-05-23T10:50:09+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -333,7 +333,7 @@
     <t>EnteteDocument.patient</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/Patient
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/PatientUsager
 </t>
   </si>
   <si>

</xml_diff>